<commit_message>
feat: finalize UX/backend flow and clean runtime artifacts
</commit_message>
<xml_diff>
--- a/data/personnel.xlsx
+++ b/data/personnel.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,41 +425,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>person_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>full_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>department</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>gender</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>rank</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>מזהה</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>שם מלא</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>זירה</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>מגדר</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>דרגה</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1001</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -456,25 +466,23 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Exec</t>
+          <t>הנהלה</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>סמנכ"ל</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>1002</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -483,25 +491,23 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Exec</t>
+          <t>הנהלה</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>סמנכ"ל</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1003</t>
-        </is>
+      <c r="A4" t="n">
+        <v>1003</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -510,25 +516,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Exec</t>
+          <t>הנהלה</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>סמנכ"ל</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1004</t>
-        </is>
+      <c r="A5" t="n">
+        <v>1004</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -537,25 +541,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Exec</t>
+          <t>הנהלה</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>סמנכ"ל</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
+      <c r="A6" t="n">
+        <v>2001</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -564,25 +566,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2002</t>
-        </is>
+      <c r="A7" t="n">
+        <v>2002</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -591,25 +591,23 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
+      <c r="A8" t="n">
+        <v>2003</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -618,25 +616,23 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2004</t>
-        </is>
+      <c r="A9" t="n">
+        <v>2004</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -645,25 +641,23 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2005</t>
-        </is>
+      <c r="A10" t="n">
+        <v>2005</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -672,25 +666,23 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2006</t>
-        </is>
+      <c r="A11" t="n">
+        <v>2006</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -699,2987 +691,2020 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
+      <c r="A12" t="n">
+        <v>2011</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>שמעון דהן</t>
+          <t>בנימין שמש</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2008</t>
-        </is>
+      <c r="A13" t="n">
+        <v>2012</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>דינה אברמוב</t>
+          <t>תמר אלון</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל בכיר</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
+      <c r="A14" t="n">
+        <v>3001</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>אליהו נחום</t>
+          <t>נתן ברק</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
+      <c r="A15" t="n">
+        <v>3002</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>חנה רוזנברג</t>
+          <t>יעל עמר</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="A16" t="n">
+        <v>3003</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>בנימין שמש</t>
+          <t>עמוס ריבלין</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
+      <c r="A17" t="n">
+        <v>3004</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>תמר אלון</t>
+          <t>נעמי שפירא</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>3001</t>
-        </is>
+      <c r="A18" t="n">
+        <v>3005</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>נתן ברק</t>
+          <t>גדעון צור</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>3002</t>
-        </is>
+      <c r="A19" t="n">
+        <v>3006</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>יעל עמר</t>
+          <t>רונית הרצוג</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>3003</t>
-        </is>
+      <c r="A20" t="n">
+        <v>3011</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>עמוס ריבלין</t>
+          <t>רועי גרינברג</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>3004</t>
-        </is>
+      <c r="A21" t="n">
+        <v>3012</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>נעמי שפירא</t>
+          <t>הדר פלד</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>3005</t>
-        </is>
+      <c r="A22" t="n">
+        <v>3013</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>גדעון צור</t>
+          <t>תומר שגב</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>3006</t>
-        </is>
+      <c r="A23" t="n">
+        <v>3014</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>רונית הרצוג</t>
+          <t>ליאת מור</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>3007</t>
-        </is>
+      <c r="A24" t="n">
+        <v>3015</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>אורי קפלן</t>
+          <t>אלעד זיו</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>3008</t>
-        </is>
+      <c r="A25" t="n">
+        <v>3016</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>מיכל וולף</t>
+          <t>קרן גל</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>3009</t>
-        </is>
+      <c r="A26" t="n">
+        <v>3021</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>איתן סגל</t>
+          <t>אסף טל</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>3010</t>
-        </is>
+      <c r="A27" t="n">
+        <v>3022</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>שירי אלבז</t>
+          <t>עינב לב</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>3011</t>
-        </is>
+      <c r="A28" t="n">
+        <v>3023</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>רועי גרינברג</t>
+          <t>יונתן הר</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>3012</t>
-        </is>
+      <c r="A29" t="n">
+        <v>4001</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>הדר פלד</t>
+          <t>אדם אור</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>3013</t>
-        </is>
+      <c r="A30" t="n">
+        <v>4002</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>תומר שגב</t>
+          <t>נועה שמיר</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>3014</t>
-        </is>
+      <c r="A31" t="n">
+        <v>4003</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ליאת מור</t>
+          <t>רון יוסף</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>3015</t>
-        </is>
+      <c r="A32" t="n">
+        <v>4004</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>אלעד זיו</t>
+          <t>מאיה דוד</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>3016</t>
-        </is>
+      <c r="A33" t="n">
+        <v>4005</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>קרן גל</t>
+          <t>עמית חיים</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>3017</t>
-        </is>
+      <c r="A34" t="n">
+        <v>4006</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ניר שרון</t>
+          <t>הילה משה</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>3018</t>
-        </is>
+      <c r="A35" t="n">
+        <v>4007</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>אפרת נוי</t>
+          <t>ליאם יעקב</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>3019</t>
-        </is>
+      <c r="A36" t="n">
+        <v>4008</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>עדי רם</t>
+          <t>תמר שרה</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>3020</t>
-        </is>
+      <c r="A37" t="n">
+        <v>4009</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>דנה ארז</t>
+          <t>אור מלכי</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>3021</t>
-        </is>
+      <c r="A38" t="n">
+        <v>4010</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>אסף טל</t>
+          <t>שקד רחל</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>3022</t>
-        </is>
+      <c r="A39" t="n">
+        <v>4011</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>עינב לב</t>
+          <t>איתי אלי</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>3023</t>
-        </is>
+      <c r="A40" t="n">
+        <v>4012</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>יונתן הר</t>
+          <t>אורי רבקה</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>3024</t>
-        </is>
+      <c r="A41" t="n">
+        <v>4021</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>שלי דר</t>
+          <t>לביא ראובן</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>4001</t>
-        </is>
+      <c r="A42" t="n">
+        <v>4022</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>אדם אור</t>
+          <t>גלי יהודית</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>4002</t>
-        </is>
+      <c r="A43" t="n">
+        <v>4023</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>נועה שמיר</t>
+          <t>עידו שמעון</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>4003</t>
-        </is>
+      <c r="A44" t="n">
+        <v>4024</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>רון יוסף</t>
+          <t>רותם אביגיל</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>4004</t>
-        </is>
+      <c r="A45" t="n">
+        <v>4025</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>מאיה דוד</t>
+          <t>שחר לוי</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>4005</t>
-        </is>
+      <c r="A46" t="n">
+        <v>4026</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>עמית חיים</t>
+          <t>אלה כהן</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>4006</t>
-        </is>
+      <c r="A47" t="n">
+        <v>4031</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>הילה משה</t>
+          <t>סהר אזולאי</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>4007</t>
-        </is>
+      <c r="A48" t="n">
+        <v>4032</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ליאם יעקב</t>
+          <t>דר מזרחי</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>4008</t>
-        </is>
+      <c r="A49" t="n">
+        <v>4033</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>תמר שרה</t>
+          <t>אלון ביטון</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>4009</t>
-        </is>
+      <c r="A50" t="n">
+        <v>4034</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>אור מלכי</t>
+          <t>עמליה גולן</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>4010</t>
-        </is>
+      <c r="A51" t="n">
+        <v>4035</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>שקד רחל</t>
+          <t>ניב מלכה</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>4011</t>
-        </is>
+      <c r="A52" t="n">
+        <v>4036</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>איתי אלי</t>
+          <t>מעיין רוזן</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>4012</t>
-        </is>
+      <c r="A53" t="n">
+        <v>4041</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>אורי רבקה</t>
+          <t>יהל אביב</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>4013</t>
-        </is>
+      <c r="A54" t="n">
+        <v>4042</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>יובל שאול</t>
+          <t>ליה גפן</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>4014</t>
-        </is>
+      <c r="A55" t="n">
+        <v>4043</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>עדן לאה</t>
+          <t>אריאל שדה</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>4015</t>
-        </is>
+      <c r="A56" t="n">
+        <v>4044</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>דניאל גד</t>
+          <t>שני ירון</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>4016</t>
-        </is>
+      <c r="A57" t="n">
+        <v>4045</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>נגה דבורה</t>
+          <t>עומר הראל</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>4017</t>
-        </is>
+      <c r="A58" t="n">
+        <v>4046</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ארי נפתלי</t>
+          <t>נופר קדם</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>4018</t>
-        </is>
+      <c r="A59" t="n">
+        <v>4047</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ליבי חנה</t>
+          <t>דור אילן</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>4019</t>
-        </is>
+      <c r="A60" t="n">
+        <v>4048</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>נדב זבולון</t>
+          <t>יסמין ברוש</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>4020</t>
-        </is>
+      <c r="A61" t="n">
+        <v>4049</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>שיר מרים</t>
+          <t>גיל ערמון</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>4021</t>
-        </is>
+      <c r="A62" t="n">
+        <v>4050</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>לביא ראובן</t>
+          <t>דניאלה אלה</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>4022</t>
-        </is>
+      <c r="A63" t="n">
+        <v>4051</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>גלי יהודית</t>
+          <t>שי דקל</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>4023</t>
-        </is>
+      <c r="A64" t="n">
+        <v>4052</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>עידו שמעון</t>
+          <t>מור תדהר</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>4024</t>
-        </is>
+      <c r="A65" t="n">
+        <v>4053</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>רותם אביגיל</t>
+          <t>ניתאי זית</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>4025</t>
-        </is>
+      <c r="A66" t="n">
+        <v>4054</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>שחר לוי</t>
+          <t>רוני ורד</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>4026</t>
-        </is>
+      <c r="A67" t="n">
+        <v>4055</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>אלה כהן</t>
+          <t>בן אורן</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>4027</t>
-        </is>
+      <c r="A68" t="n">
+        <v>4056</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ים פרץ</t>
+          <t>תהל שקד</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>4028</t>
-        </is>
+      <c r="A69" t="n">
+        <v>4057</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>צוף חדד</t>
+          <t>אייל רימון</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>4029</t>
-        </is>
+      <c r="A70" t="n">
+        <v>4058</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>טל דהן</t>
+          <t>יערה הדס</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>4030</t>
-        </is>
+      <c r="A71" t="n">
+        <v>4071</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ענבר שלום</t>
+          <t>נהוראי כרמל</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>4031</t>
-        </is>
+      <c r="A72" t="n">
+        <v>4072</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>סהר אזולאי</t>
+          <t>סיון גולני</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>4032</t>
-        </is>
+      <c r="A73" t="n">
+        <v>4073</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>דר מזרחי</t>
+          <t>יניב הרמון</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>4033</t>
-        </is>
+      <c r="A74" t="n">
+        <v>4074</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>אלון ביטון</t>
+          <t>לירון תבור</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>4034</t>
-        </is>
+      <c r="A75" t="n">
+        <v>4075</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>עמליה גולן</t>
+          <t>אמיר כנרת</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>4035</t>
-        </is>
+      <c r="A76" t="n">
+        <v>4076</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ניב מלכה</t>
+          <t>רננה ירדן</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>4036</t>
+          <t>5001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>מעיין רוזן</t>
+          <t>יובל הדר</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>הנהלה</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>4037</t>
+          <t>5002</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>נועם אברמוב</t>
+          <t>הילה קשת</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>הנהלה</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>4038</t>
+          <t>5003</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>אגם נחום</t>
+          <t>עומר בן דוד</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>4039</t>
+          <t>5004</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>בראל שמש</t>
+          <t>רות לביא</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>5005</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>חן אלון</t>
+          <t>איתי שלו</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>מו"פ</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>4041</t>
+          <t>5006</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>יהל אביב</t>
+          <t>שני רותם</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>4042</t>
+          <t>5007</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ליה גפן</t>
+          <t>טל ברעם</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מכירות</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>4043</t>
+          <t>5008</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>אריאל שדה</t>
+          <t>מיקה דביר</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>4044</t>
+          <t>5009</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>שני ירון</t>
+          <t>רון כפיר</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>מערכות מידע</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>4045</t>
+          <t>5010</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>עומר הראל</t>
+          <t>אורית סלע</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>בקרת איכות</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>4046</t>
+          <t>5011</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>נופר קדם</t>
+          <t>גל עמרם</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>בקרת איכות</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>4047</t>
+          <t>5012</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>דור אילן</t>
+          <t>ליה שמאי</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>תפעול</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>מנהל</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>4048</t>
+          <t>5013</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>יסמין ברוש</t>
+          <t>ניר תבור</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>תפעול</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>בנים</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>4049</t>
+          <t>5014</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>גיל ערמון</t>
+          <t>אביגיל סער</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>תפעול</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>בנות</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>4050</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>דניאלה אלה</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>4051</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>שי דקל</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>4052</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>מור תדהר</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>4053</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>ניתאי זית</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>4054</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>רוני ורד</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>4055</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>בן אורן</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>4056</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>תהל שקד</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>4057</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>אייל רימון</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>4058</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>יערה הדס</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>4059</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>מתן זמיר</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>4060</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>אביה צבר</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>4061</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>ליעד ארז</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>4062</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>הדס ענבל</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>4063</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>עילאי נריה</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>4064</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>נוגה ליבנה</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>4065</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>אופיר גדי</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>4066</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>ליאן נעמה</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>4067</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>רז עמית</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>4068</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>טליה שגיא</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>4069</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>אלעד נצר</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>4070</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>עדי חורש</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>4071</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>נהוראי כרמל</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>R&amp;D</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>4072</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>סיון גולני</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>R&amp;D</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>4073</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>יניב הרמון</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>4074</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>לירון תבור</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>4075</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>אמיר כנרת</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>4076</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>רננה ירדן</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>4077</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>עידן נגב</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>4078</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>אילנה גליל</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>4079</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>תמיר ערבה</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Junior</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>4080</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>אורלי חרמון</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Junior</t>
+          <t>זוטר</t>
         </is>
       </c>
     </row>

</xml_diff>